<commit_message>
Update media links Excel with 16 more links (15 posts), dates where decodable
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B6RPWkBpLKoctTdaNtAabD
</commit_message>
<xml_diff>
--- a/Media_Links_Details.xlsx
+++ b/Media_Links_Details.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Media links" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All links given" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Media links'!$A$1:$N$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Media links'!$A$1:$R$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -81,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -91,6 +92,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -461,26 +465,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="48" customWidth="1" min="12" max="12"/>
-    <col width="52" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="52" customWidth="1" min="15" max="15"/>
+    <col width="56" customWidth="1" min="16" max="16"/>
+    <col width="42" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" customHeight="1">
+    <row r="1" ht="44" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>#</t>
@@ -488,65 +496,85 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Link (as given)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Also given as (same post)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>City / District</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>State / Region</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>How the state was identified</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Posted by (page)</t>
-        </is>
-      </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Post page address</t>
+          <t>How city and state were identified</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Posted by (page or account)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Post address</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Posted date</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Where the date came from</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Ceremony date in report (not the posting date)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Views (at check)</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Reactions (at check)</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Caption (Somali, as posted)</t>
-        </is>
-      </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Views</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Reactions</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Caption (original language)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>Caption (English, translated)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Checked on</t>
         </is>
@@ -556,67 +584,79 @@
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>https://www.facebook.com/reel/3743534559129368</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1PzbeCmK6u/</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Cadaado</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Galmudug</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Inferred from city (Cadaado is in Galmudug); the caption names the city only</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Telefishinka Qaranka Soomaaliyeed</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/sntvnews/videos/haweenka-ka-ganacsada-caanaha-xoolaha-ee-magaalada-cadaado-ayaa-lagu-taageeray-q/3743534559129368/</t>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>City named in caption; state inferred from the city (Cadaado is in Galmudug)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
+          <t>Telefishinka Qaranka Soomaaliyeed (SNTV)</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/sntvnews/videos/3743534559129368/</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>Not shown by Facebook to logged-out visitors</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>18 Aug 2026</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>6K</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>61</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>Haweenka ka ganacsada caanaha xoolaha ee magaalada Cadaado ayaa lagu taageeray qalab qaboojiyeyaal ah oo ku shaqeeya cadceedda.</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Women who trade in livestock milk in Cadaado town were supported with solar-powered refrigeration equipment.</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>14 Oct 2026</t>
         </is>
@@ -626,67 +666,79 @@
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>https://www.facebook.com/reel/2053184808633587</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/reel/2053184808633587 (given 3 times); https://www.facebook.com/share/v/18Thwu3VLX/</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Galkacyo</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Galmudug</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Caption names the Galmudug Ministry of Livestock</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Telefishinka Qaranka Soomaaliyeed</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/sntvnews/videos/wasaaradda-xanaanada-xoolaha-galmudug-oo-kaashanaysa-wasaaradda-xanaaanada-xoola/2053184808633587/</t>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Caption names Galkacyo and the Galmudug Ministry of Livestock</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
+          <t>Telefishinka Qaranka Soomaaliyeed (SNTV)</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/sntvnews/videos/2053184808633587/</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
           <t>Not shown by Facebook to logged-out visitors</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>18 Aug 2026</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>14K</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>127</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>Wasaaradda Xanaanada Xoolaha Galmudug oo kaashanaysa Wasaaradda Xanaaanada Xoolaha DFS ayaa agab ganacsi u qaybisay qaar ka mid ah haweenka ka ganacsada caanaha ee ku nool Gaalkacyo.</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>The Galmudug Ministry of Livestock, in cooperation with the Federal (DFS) Ministry of Livestock, distributed business equipment to some of the women milk traders living in Galkacyo.</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr">
         <is>
           <t>14 Oct 2026</t>
         </is>
@@ -696,67 +748,79 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>https://www.facebook.com/reel/916665714471740</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Mogadishu</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Banadir</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Caption names the Banadir Regional Administration</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Telefishinka Qaranka Soomaaliyeed</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/sntvnews/videos/guddoomiye-ku-xigeenka-arimaha-bulshada-maamulka-gobolka-banaadir-ayaa-haween-ka/916665714471740/</t>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Caption names the Banadir Regional Administration; city is Mogadishu (Banadir)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
+          <t>Telefishinka Qaranka Soomaaliyeed (SNTV)</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/sntvnews/videos/916665714471740/</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
           <t>Not shown by Facebook to logged-out visitors</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>6 Sep 2026</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>37K</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>982</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>Guddoomiye Ku-xigeenka Arimaha Bulshada Maamulka Gobolka Banaadir ayaa haween ka ganacsada caanaha ku wareejiyay qaboojiyeyaal ku shaqeeya tamarta cadceedda iyo agab loogu talagalay kaydinta iyo...</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>The Deputy Chairperson for Social Affairs of the Banadir Regional Administration handed over solar-powered refrigerators and equipment for storing and preserving milk to women milk traders. (Caption is cut off on the page.)</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>The same SNTV story is also on YouTube (row 9) and TikTok (row 10).</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>14 Oct 2026</t>
         </is>
@@ -766,67 +830,83 @@
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>https://www.facebook.com/reel/1881138039767781</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1BTGkStX6h/</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Jowhar</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Hirshabelle</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Caption names Hirshabelle and the Federal Government</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Caption names Jowhar, Hirshabelle and the Federal Government</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Somali Cable TV</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/OfficialSomaliCableTV/videos/mashruuc-loogu-talagay-haweenka-caana-ku-iibiya-magaalada-jowhar-oo-lasoo-bandhi/1881138039767781/</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/OfficialSomaliCableTV/videos/1881138039767781/</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Not shown by Facebook to logged-out visitors</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>14 Sep 2026</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>9.2K</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>166</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>Mashruuc loogu talagay Haweenka Caana ku iibiya magaalada Jowhar oo lasoo bandhigay iyo Hirshabeelle &amp; Xukuumadda Federalka oo wadajir u fulinaya mashruucaasi.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>A project for women who sell milk in Jowhar town was presented, with Hirshabelle and the Federal Government implementing it jointly.</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>Same caption as row 6 (reel and post versions).</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
         <is>
           <t>14 Oct 2026</t>
         </is>
@@ -836,85 +916,868 @@
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>https://www.facebook.com/reel/4439016306360579</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1EfpjgAyyc/</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Balcad</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Hirshabelle</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Caption names the Hirshabelle Ministry of Livestock</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Telefishinka Qaranka Soomaaliyeed</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/sntvnews/videos/wasaaradda-xannaanada-xoolaha-hirshabeelle-oo-kaashaneysa-wasaaradda-xanaanada-x/4439016306360579/</t>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Caption names Balcad district and the Hirshabelle Ministry of Livestock</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
+          <t>Telefishinka Qaranka Soomaaliyeed (SNTV)</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/sntvnews/videos/4439016306360579/</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
           <t>Not shown by Facebook to logged-out visitors</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>14 Sep 2026</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>6.3K</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>68</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>Wasaaradda Xannaanada Xoolaha Hirshabeelle oo kaashaneysa Wasaaradda Xanaanada Xoolaha XFS ayaa agab loogu talo galay in kor loogu qaado ganacsiga ku wareejisay  qaar kamid ah haweenka degmada Balcad.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>The Hirshabelle Ministry of Livestock, in cooperation with the Federal (XFS) Ministry of Livestock, handed over equipment to boost the business of some women in Balcad district.</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>Second Balcad video is row 11.</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
         <is>
           <t>14 Oct 2026</t>
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Facebook (post)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1K3tPWDFY5/</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Jowhar</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Hirshabelle</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Caption names Jowhar, Hirshabelle and the Federal Government</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Somali Cable TV</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/OfficialSomaliCableTV/posts/1132613816091965/</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Not shown by Facebook to logged-out visitors</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>14 Sep 2026</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Mashruuc loogu talagay Haweenka Caana ku iibiya magaalada Jowhar oo lasoo bandhigay iyo Hirshabeelle &amp; Xukuumadda Federalka oo wadajir u fulinaya mashruucaasi.</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>A project for women who sell milk in Jowhar town was presented, with Hirshabelle and the Federal Government implementing it jointly.</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>Same video and caption as row 4, posted as a regular post. The page shows no view or reaction counts to logged-out visitors.</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>14 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1C1BYiQ3f8/</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Kismayo</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Jubaland</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Caption names Kismayo and the Jubaland Ministry of Livestock</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Radio Kismayo</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/100090329544863/videos/1371474821394160/</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Not shown by Facebook to logged-out visitors</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>30 Sep 2026</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Wasaaradda Xannaanada Xoolaha, Jubbaland, oo  magaalada Kismaayo ku qabatay munaasabad lagu taageerayo kobcinta iyo horumarinta ganacsiga caanaha ee haweenka.</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>The Jubaland Ministry of Livestock held an event in Kismayo town to support the growth and development of women's milk trade.</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>Same caption as row 8. No counts shown to logged-out visitors.</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>14 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Facebook (post)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1P8MVcn4z6/</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Kismayo</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Jubaland</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Caption names Kismayo and the Jubaland Ministry of Livestock</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Jubbaland TV</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/JLTVOFFICIAL/posts/1573603554811340/</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Not shown by Facebook to logged-out visitors</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>30 Sep 2026</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Wasaaradda Xannaanada Xoolaha, Jubbaland, oo  magaalada Kismaayo ku qabatay munaasabad lagu taageerayo kobcinta iyo horumarinta ganacsiga caanaha ee haweenka.</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>The Jubaland Ministry of Livestock held an event in Kismayo town to support the growth and development of women's milk trade.</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>Same caption as row 7.</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>14 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>https://youtu.be/r6KLf6HcRBw?si=y_cvvihn6hTwlOGP</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Mogadishu</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Banadir</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Title names the Banadir Regional Administration; city is Mogadishu (Banadir)</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Somali National Television (SNTV)</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=r6KLf6HcRBw</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Not available (YouTube blocked the check)</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>YouTube refused the request (rate limit), so the date could not be read</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>6 Sep 2026</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>Maamulka Gobolka Banaadir ayaa haween ka ganacsada caanaha ku wareejiyay agab</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>The Banadir Regional Administration handed over equipment to women milk traders.</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>Only the title could be read (from YouTube's public embed data). Open the video to read the date.</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>14 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>https://vt.tiktok.com/ZSqhyFG6W/</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Mogadishu</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Banadir</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Caption names the Banadir Regional Administration; city is Mogadishu (Banadir)</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>SNTV (@sntvnews1)</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@sntvnews1/video/7683076315645332757</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08 (about 08:20 UTC)</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Decoded from the TikTok video ID and the page's createTime; both agree</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>6 Sep 2026</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>50.4K plays</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>Guddoomiye Ku-xigeenka Arimaha Bulshada Maamulka Gobolka Banaadir ayaa haween ka ganacsada caanaha ku wareejiyay qaboojiyeyaal ku shaqeeya tamarta cadceedda iyo agab loogu talagalay kaydinta iyo ilaalinta caanaha</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>The Deputy Chairperson for Social Affairs of the Banadir Regional Administration handed over solar-powered refrigerators and equipment for storing and preserving milk to women milk traders.</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>Posted 2 days after the 6 Sep ceremony date in the report.</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>14 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1BzDfny6hy/</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Balcad</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Hirshabelle</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Caption names Balcad and the Hirshabelle Ministry of Livestock</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Telefishinka HirShabeelle</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/TvHirShabeelle/videos/1073825435055391/</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Not shown by Facebook to logged-out visitors</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>14 Sep 2026</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>2.6K</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Wasaaradaha Xannaanada Xoolaha Hirshabeelle oo Haweenka Caanaha ka Ganacsada Balcad ku wareejiyay agab muhiim u ah ganacsiga.</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>The Hirshabelle Ministries of Livestock handed over equipment important for business to women milk traders in Balcad.</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>Second Balcad video (first is row 5).</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>14 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1JpAYpvdNS/</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Dhusamareeb</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Galmudug</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Caption names Dhuusamareeb; state inferred from the city (Dhusamareeb is in Galmudug)</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Telefishinka Qaranka Soomaaliyeed (SNTV)</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/sntvnews/videos/1010232142051557/</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Not shown by Facebook to logged-out visitors</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>18 Aug 2026</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>372</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>Haweenka ka ganacsada caanaha xoolaha ee magaalada Dhuusamareeb ayaa loogu deeqay qalab qaboojiyeyaal ah oo ku shaqeeya cadceedda.</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>Women milk traders in Dhuusamareeb town were given solar-powered refrigeration equipment.</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>14 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Facebook (post)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1D4YYo3kHt/</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Dhusamareeb</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Galmudug</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Caption names Dhuusamareeb; state inferred from the city (Dhusamareeb is in Galmudug)</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Abdulahi Warsame Roble (personal profile)</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/abdulahirob/posts/1568262718015164/</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Not shown by Facebook to logged-out visitors</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>18 Aug 2026</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Haween Caanoley ah oo Dhuusamareeb lagu taageeray Qalab Qaboojiye oo Cadceed ku shaqeeya #ILASOCO</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>Milk-selling women in Dhuusamareeb were supported with solar-powered refrigeration equipment. #ILASOCO</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>A personal profile, not a news page. No counts shown to logged-out visitors.</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>14 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>https://lnkd.in/p/e4gU2_tj</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Not named (rural cities of Galmudug)</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Galmudug</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Post says the road trip was between major rural cities in Galmudug State, on a HoA DRIVE Somalia mission</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Abdulkdir Hassan (LinkedIn)</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/posts/abdulkdir-hassan-37014b135_agriconnect-share-7509325141781241856-</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 (about 18:57 UTC)</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Decoded from the LinkedIn post ID and the page's datePublished; both agree</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>"Somalia's Rural Food System Under Threat from Climate Change and Imported Foods" (English post)</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>A reflection by the author after road travel between rural cities in Galmudug on a HoA DRIVE Somalia mission about women in the dairy value chain, then on imported food, local production and climate effects.</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>This is a general reflection, not a post about a handover ceremony. No ceremony date applies. Check whether it belongs in your media list.</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>14 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Facebook (story)</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>https://m.facebook.com/story.php?story_fbid=pfbid02L9xoCahkAkqwzjpUoh3iJBhbuvwKQzBfRpTb5pZG5B5VuCrLKRe2qGty9xrp2rFbl&amp;id=100064851304084&amp;sfnsn=wa&amp;mibextid=6aamW6</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Could not be read</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Could not be read</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Facebook asks for a login, so the post content is hidden</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Page ID 100064851304084 (name not visible)</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Not shown by Facebook to logged-out visitors</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>Not readable without logging in. Send a screenshot or the caption and I will fill in this row.</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>14 Oct 2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N6"/>
+  <autoFilter ref="A1:R16"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -926,58 +1789,578 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Link (exactly as given)</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Opened?</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Same post as row (Media links sheet)</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/reel/3743534559129368</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Earlier list</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/reel/2053184808633587</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Earlier list</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/reel/916665714471740</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Earlier list</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/reel/1881138039767781</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Earlier list</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/reel/4439016306360579</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Earlier list</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1K3tPWDFY5/</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1EfpjgAyyc/</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Share link to the Balcad video already in row 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/r6KLf6HcRBw?si=y_cvvihn6hTwlOGP</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Title only</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>YouTube blocked the page, so no date</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1PzbeCmK6u/?mibextid=wwXIfr</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Share link to the Cadaado video already in row 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/reel/2053184808633587</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Duplicate: Galkacyo video, already in the earlier list</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/reel/2053184808633587</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Duplicate: given twice in this list</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1C1BYiQ3f8/</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1P8MVcn4z6/</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>https://m.facebook.com/story.php?story_fbid=pfbid02L9xoCahkAkqwzjpUoh3iJBhbuvwKQzBfRpTb5pZG5B5VuCrLKRe2qGty9xrp2rFbl&amp;id=100064851304084&amp;sfnsn=wa&amp;mibextid=6aamW6</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>No (login required)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Needs a login</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>https://lnkd.in/p/e4gU2_tj</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1BTGkStX6h/</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Share link to the Jowhar video already in row 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1BzDfny6hy/</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>https://vt.tiktok.com/ZSqhyFG6W/</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1JpAYpvdNS/</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/1D4YYo3kHt/</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/v/18Thwu3VLX/</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Share link to the Galkacyo video already in row 2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="130" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
           <t>How this sheet was made</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Each link was opened without logging in. City, state, page name, caption, views and reactions come from the public page.</t>
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Each link was opened without logging in. City, state, page name, caption and counts come from the public page.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Posted date: Facebook does not show the posting date to logged-out visitors, so it is left as not available. Add it by hand from each post if you need it.</t>
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>22 links were given in total (5 earlier, 17 new counting the repeats). They resolve to 15 different posts, listed in the Media links sheet. The All links given sheet shows where each link went.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Ceremony date: this is the handover date from the Rasmi reports, shown only for comparison. It is not the date the video was posted.</t>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Posted date: Facebook does not show the posting date to logged-out visitors. YouTube blocked the check. The two dates shown (TikTok 8 Sep 2026, LinkedIn 25 Sep 2026) were decoded from the post IDs and agree with a date in the page.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Views and reactions are a snapshot on the check date and will change.</t>
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>To fill the Facebook and YouTube dates, send the dates from the posts or screenshots.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Ceremony date: the handover date in the Rasmi reports, shown only for comparison. It is not the date the video was posted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>City and state: taken from the caption where it names one. Where only the city is named, the state is inferred from the city, and the row says so.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Views and reactions are a snapshot on the check date and will change. Some pages show no counts to logged-out visitors, so those cells are blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>English captions are a translation from Somali for convenience. Check them before using them in a report.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>State is taken from the caption where it names one. Cadaado is the only row where the state is inferred from the city.</t>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Row 14 (LinkedIn) is a general reflection post about a Galmudug mission, not a handover post. Row 15 could not be read without a login.</t>
         </is>
       </c>
     </row>

</xml_diff>